<commit_message>
docs: consolidate learning review materials and cards
Backfill Triton study logs and authorized visible-dialogue archives, restore message references, and add a shared review index.

Refresh five managed Markji sets to 63 cards on template 1.1.0, record verified uploads, and update the repository overview.

Validation: staged whitespace check, skill materialization check, and managed artifact verification passed (5 sets, 63 cards, 15 XLSX workbooks).
</commit_message>
<xml_diff>
--- a/docs/algorithm-interview-learning/cards/algorithm-interview-lesson-01-constraint-driven-selection-correction.xlsx
+++ b/docs/algorithm-interview-learning/cards/algorithm-interview-lesson-01-constraint-driven-selection-correction.xlsx
@@ -9,7 +9,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -41,119 +41,90 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">完整说明 Two Sum 双层枚举基线</t>
+          <t xml:space="preserve">为什么只数循环层数还不够？</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t xml:space="preserve">用 i &lt; j 枚举两个不同下标</t>
+          <t xml:space="preserve">解释 Two Sum 的 i &lt; j 双层枚举基线</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t xml:space="preserve">先证明 i &lt; j 完整覆盖，再说明工作量与重复查询。</t>
+          <t xml:space="preserve">还要说明覆盖范围、比较次数和重复工作。</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t xml:space="preserve">第一个 n 在外层，第二个 n 在内层。</t>
+          <t xml:space="preserve">第一个 n 在哪里，第二个 n 在哪里</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t xml:space="preserve">[T#B,!36b59d#结论]：基线说明要同时交代完整性、成本来源和瓶颈。
-• [T#B#完整性]：i &lt; j 恰好覆盖每个不同下标的无序组合。
-• [T#B#工作量]：比较次数为 n(n−1)/2，因此是 Θ(n²)。
-• [T#B#瓶颈]：对补数是否存在的查询被重复执行，优化应优先减少这类重复工作。
-[T#B,!c47f17#边界]：只数循环层数既不能证明解空间完整，也不能定位可优化瓶颈。</t>
+          <t xml:space="preserve">[T#B,!36b59d#结论]：用解空间 → 成本 → 瓶颈说明基线。
+• [T#B#覆盖]：i &lt; j 恰好枚举每个不同下标的无序组合。
+• [T#B#成本]：共有 n(n−1)/2 对，比较工作量为 Θ(n²)。
+• [T#B#瓶颈]：反复查找补数是否存在，是可继续考察的重复工作。
+[T#B,!c47f17#边界]：数出两层循环，不等于证明枚举完整或找到了可优化的重复工作。</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t xml:space="preserve">判断候选方向受阻后能得出多强的结论</t>
+          <t xml:space="preserve">候选都受阻，能断言无法优化吗？</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t xml:space="preserve">只读输入和 O(1) 额外空间排除了保存历史与排序</t>
+          <t xml:space="preserve">只读输入与 O(1) 额外空间排除了排序和保存历史</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t xml:space="preserve">只能说这些候选不满足约束，当前尚未找到有效优化。</t>
+          <t xml:space="preserve">只能说当前检查的候选不满足约束。</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t xml:space="preserve">目前就没有满足所有条件的优化方案了。</t>
+          <t xml:space="preserve">目前就没有满足所有条件的优化方案了</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t xml:space="preserve">[T#B,!36b59d#结论]：排除有限候选不等于证明所有优化不存在。
-• [T#B#可陈述]：已检查哪些方向、它们违反什么约束、当前最强可行结论是什么。
-• [T#B#继续确认]：是否还有可利用的数据结构、值域、顺序或访问模型。
-[T#B,!c47f17#边界]：宣称无更优解或最优性，需要明确计算模型下的下界证明。</t>
+          <t xml:space="preserve">[T#B,!36b59d#结论]：排除有限候选，不能证明所有优化都不存在。
+• [T#B#已知]：说明检查了哪些方案，各违反哪项约束。
+• [T#B#未知]：保留尚未探索的值域、顺序或访问条件。
+[T#B,!c47f17#边界]：宣称不存在更优方案，需要相应计算模型下的下界论证。</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">判断既有基线在新访问模型下是否可执行</t>
+          <t xml:space="preserve">元素值域能直接限制 target 吗？</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t xml:space="preserve">精确判重从随机访问数组改为单遍数据流</t>
+          <t xml:space="preserve">Two Sum 的元素只来自 {0,1,2}</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t xml:space="preserve">先检查基线依赖的回看、随机访问或多遍读取是否仍可用。</t>
+          <t xml:space="preserve">只有保证有解，才能推出 target 属于 0 到 4。</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t xml:space="preserve">数组上的 O(n²) 双层枚举仍可直接作为单遍流基线。</t>
+          <t xml:space="preserve">target 也只可能有 0、1、2、3、4……共 5 种情况</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t xml:space="preserve">[T#B,!36b59d#结论]：算法在新输入表示下必须先满足可执行性，才谈复杂度。
-• [T#B#原有依赖]：数组双层枚举需要回看或随机访问已见元素。
-[T#B,!c47f17#边界]：单遍流中已消费元素不可重新枚举，所以该数组基线不能直接迁移。</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">判断固定元素值域能否限制 Two Sum 的 target</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">nums 的元素只来自 {0,1,2}</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">值域只限定可达和值；保证存在解时才能推出 target 在 0 到 4。</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">target 也只可能有 0、1、2、3、4。</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">[T#B,!36b59d#结论]：元素值域约束的是可达和值，不是所有合法 target。
-• [T#B#有解保证]：若题目保证存在解，target 必须是两个元素的和值，因此落在 0 到 4。
-[T#B,!c47f17#边界]：若不保证有解且没有其他 target 约束，target 可以在范围外，此时无解。</t>
+          <t xml:space="preserve">[T#B,!36b59d#结论]：元素值域限制可达和值，不自动限制所有合法输入 target。
+• [T#B#有解保证]：两个元素的和值必落在 0 到 4，故有解时 target 也在其中。
+[T#B,!c47f17#边界]：没有有解保证或额外 target 约束时，范围外的 target 可以合法，只是没有解。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: clarify review cards and add lesson previews
Make all 113 cards across Triton lessons 01-06 and algorithm lesson 01 self-contained while preserving their knowledge targets, identities, sources, and original error quotes. Refresh 21 XLSX files and add per-lesson Markdown previews with navigation.

Validation: all seven memo-cards requests verified as no-op with no artifact drift; all cards active; preview counts and 505 links checked. Keep the agent-skills submodule pointer at de52504.
</commit_message>
<xml_diff>
--- a/docs/algorithm-interview-learning/cards/algorithm-interview-lesson-01-constraint-driven-selection-correction.xlsx
+++ b/docs/algorithm-interview-learning/cards/algorithm-interview-lesson-01-constraint-driven-selection-correction.xlsx
@@ -41,17 +41,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">为什么只数循环层数还不够？</t>
+          <t xml:space="preserve">向面试官解释 Two Sum：给定长度为 n 的数组 nums 和目标值 target，要找两个不同原下标，使对应元素之和等于 target。怎样把双层枚举基线的覆盖、成本和瓶颈讲清楚，而不只说它有两层循环？</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t xml:space="preserve">解释 Two Sum 的 i &lt; j 双层枚举基线</t>
+          <t xml:space="preserve">数组允许重复访问；基线固定第一个下标，再检查它后面的每个下标，找到符合要求的一对即可返回。</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t xml:space="preserve">还要说明覆盖范围、比较次数和重复工作。</t>
+          <t xml:space="preserve">说明每个不同下标对为何恰好被检查一次，再由比较次数得到最坏成本，最后指出对补数存在性的重复查询。</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -61,28 +61,30 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t xml:space="preserve">[T#B,!36b59d#结论]：用解空间 → 成本 → 瓶颈说明基线。
-• [T#B#覆盖]：i &lt; j 恰好枚举每个不同下标的无序组合。
-• [T#B#成本]：共有 n(n−1)/2 对，比较工作量为 Θ(n²)。
-• [T#B#瓶颈]：反复查找补数是否存在，是可继续考察的重复工作。
-[T#B,!c47f17#边界]：数出两层循环，不等于证明枚举完整或找到了可优化的重复工作。</t>
+          <t xml:space="preserve">[T#B,!36b59d#结论]：双层枚举的解释应连起三个问题：为什么不会漏解、为什么最坏需要平方级工作量，以及哪些重复工作值得尝试消除。
+• [T#B#覆盖]：外层下标 i 固定第一个元素，内层下标 j 只遍历其后的元素。任意两个不同下标都有唯一的较小者和较大者，因此所有合法无序下标对都会恰好出现一次；既不复用同一元素，也不把交换顺序后的同一对重复计算。
+[E##0\le i&lt;j&lt;n,\qquad \mathrm{nums}_i+\mathrm{nums}_j=\mathrm{target}]
+• [T#B#成本]：外层每前进一步，后面可配对的元素就少一个。若必须检查完全部候选，比较次数是从 n−1 到 1 的和；在每次取值、相加和比较为常数成本的前提下，这给出平方级最坏时间。
+[E##\sum_{i=0}^{n-2}(n-1-i)=\frac{n(n-1)}{2}=\Theta(n^2)]
+• [T#B#瓶颈]：每固定一个元素，都要重新扫描候选位置，查找“target 减去该元素”这个补数是否存在。下一步应验证：能否利用允许的额外状态、值域或顺序减少这些重复查询，同时仍满足原下标和互异下标要求。
+[T#B,!c47f17#边界]：找到答案可以提前返回，因此某次输入不一定做完全部比较。仅数出两层循环，既没有证明覆盖完整，也没有证明存在符合题目约束的优化。</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t xml:space="preserve">候选都受阻，能断言无法优化吗？</t>
+          <t xml:space="preserve">为只读数组上的 Two Sum 寻找更快方案，题目只允许常数额外空间；检查过的排序方案和保存历史方案都违反约束。此时能否断言不存在比双层枚举更好的算法，应该怎样表述结论？</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t xml:space="preserve">只读输入与 O(1) 额外空间排除了排序和保存历史</t>
+          <t xml:space="preserve">需要找出和值等于 target 的两个不同原下标；目前排除的只是会重排原数组的排序方案，以及存储量随输入规模增长的历史保存方案。</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t xml:space="preserve">只能说当前检查的候选不满足约束。</t>
+          <t xml:space="preserve">只能说这些已检查的候选不满足约束，目前尚未找到有效优化；不能由此断言所有优化都不存在。</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -92,27 +94,28 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t xml:space="preserve">[T#B,!36b59d#结论]：排除有限候选，不能证明所有优化都不存在。
-• [T#B#已知]：说明检查了哪些方案，各违反哪项约束。
-• [T#B#未知]：保留尚未探索的值域、顺序或访问条件。
-[T#B,!c47f17#边界]：宣称不存在更优方案，需要相应计算模型下的下界论证。</t>
+          <t xml:space="preserve">[T#B,!36b59d#结论]：“当前候选受阻”是有限检查的结果；“不存在更优算法”是对所有允许算法的断言，两者所需证据不同。
+• [T#B#已知证据]：把被排除的具体方案与约束对应起来：直接重排原数组违反只读要求，保存随输入增多的历史记录违反常数额外空间要求。不要把某个方案被排除扩大成整个思路类别一律不可用。
+• [T#B#仍待检查]：继续区分尚未确认或利用的条件，例如值域是否固定、输入是否已有顺序、允许怎样访问。固定小值域就可能重新允许固定大小的状态，所以两个常见方案失败并没有穷尽所有可能。
+• [T#B#可用表述]：可以说：“我目前检查的这两个方案分别违反只读和空间约束，暂时没有找到满足全部条件的优化；接下来需要核对值域、顺序和访问条件。”
+[T#B,!c47f17#边界]：要宣称双层枚举已经最优，或不存在更快方案，需要在明确的输入条件和计算模型下给出相应下界论证；“我暂时想不到”不能替代证明。</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">元素值域能直接限制 target 吗？</t>
+          <t xml:space="preserve">Two Sum 要求在数组中选两个不同下标，使其元素和等于给定 target；已知每个元素只能是 0、1、2。仅凭这个值域，能否断言合法输入的 target 只能是 0 到 4？</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Two Sum 的元素只来自 {0,1,2}</t>
+          <t xml:space="preserve">需要区分“两个元素能够得到的和值范围”与“题目允许传入的 target 范围”，并检查题目是否保证有解。</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t xml:space="preserve">只有保证有解，才能推出 target 属于 0 到 4。</t>
+          <t xml:space="preserve">仅凭元素值域，只能限制可达和值；再有“保证存在一对解”的前提，才能由此推出 target 在 0 到 4 内。</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -122,9 +125,11 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t xml:space="preserve">[T#B,!36b59d#结论]：元素值域限制可达和值，不自动限制所有合法输入 target。
-• [T#B#有解保证]：两个元素的和值必落在 0 到 4，故有解时 target 也在其中。
-[T#B,!c47f17#边界]：没有有解保证或额外 target 约束时，范围外的 target 可以合法，只是没有解。</t>
+          <t xml:space="preserve">[T#B,!36b59d#结论]：元素值域约束的是两数相加可能产生什么结果，不会自动把范围之外的 target 变成非法输入。
+• [T#B#推导前提]：两个元素都只能取 0、1、2，因此任意一对的和值只能落在 0 到 4。若题目保证有解，target 必须等于其中某对的和值，才可据此限制 target。
+[E##\mathrm{nums}_i,\mathrm{nums}_j\in\{0,1,2\}\quad\Longrightarrow\quad 0\le\mathrm{nums}_i+\mathrm{nums}_j\le4]
+• [T#B#范围外例子]：例如题目没有限制 target、也没有保证有解时，传入 target 为 5 与元素值域并不矛盾；这个输入只是不存在符合要求的一对元素。
+[T#B,!c47f17#边界]：target 落在 0 到 4 内也不保证当前数组有解，还要看实际有哪些元素，以及能否使用两个不同下标。若题目另行规定 target 范围，则应依据那条明确约束。</t>
         </is>
       </c>
     </row>

</xml_diff>